<commit_message>
Clean up the 23 flagged workbook entries (database revision 3)
The plausibility ranges added in 1.3.2 flagged 23 entries. Twenty-two
were placeholder zeros in "Max Print Speed", which the generator already
stored as "not specified" — blanking those cells changes nothing in the
generated JSON, it only stops the warnings. The twenty-third was a real
error: a printer listed at 300 mm3/s of volumetric flow, roughly ten
times what any hotend can manage, corrected to 15.

Bumps dataRevision to 3. The v1.3.2 build ships revision 2 with that
flow field null, so leaving the number alone would put two different
datasets under the same revision — exactly the ambiguity the refresh
prompt exists to resolve, and unfixable once 1.3.2 is published.

Only that one printer's owners see a refresh prompt from this, since
specChangesForProfile surfaces a profile only when a value actually
differs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Printer_Database/Printer_Database.xlsx
+++ b/Printer_Database/Printer_Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prsda\Desktop\Printer_Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prsda\Documents\GitHub\Filament_Calibration_Wizard\Printer_Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B89EC8-89C0-4913-8738-7846356B81BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B636187F-1C9B-4317-A728-97DD177926A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Printer Specifications" sheetId="1" r:id="rId1"/>
@@ -9833,9 +9833,7 @@
       <c r="N106" s="2">
         <v>165</v>
       </c>
-      <c r="O106" s="2">
-        <v>7000</v>
-      </c>
+      <c r="O106" s="2"/>
       <c r="P106" s="2">
         <v>7000</v>
       </c>
@@ -14065,7 +14063,7 @@
         <v>27</v>
       </c>
       <c r="I177" s="4">
-        <v>300</v>
+        <v>15</v>
       </c>
       <c r="J177" s="4" t="s">
         <v>444</v>
@@ -22599,9 +22597,7 @@
       <c r="N316" s="2">
         <v>420</v>
       </c>
-      <c r="O316" s="2">
-        <v>0</v>
-      </c>
+      <c r="O316" s="2"/>
       <c r="P316" s="2">
         <v>2000</v>
       </c>
@@ -22658,9 +22654,7 @@
       <c r="N317" s="4">
         <v>400</v>
       </c>
-      <c r="O317" s="4">
-        <v>0</v>
-      </c>
+      <c r="O317" s="4"/>
       <c r="P317" s="4">
         <v>4500</v>
       </c>
@@ -22717,9 +22711,7 @@
       <c r="N318" s="2">
         <v>420</v>
       </c>
-      <c r="O318" s="2">
-        <v>0</v>
-      </c>
+      <c r="O318" s="2"/>
       <c r="P318" s="2">
         <v>4500</v>
       </c>
@@ -22776,9 +22768,7 @@
       <c r="N319" s="4">
         <v>420</v>
       </c>
-      <c r="O319" s="4">
-        <v>0</v>
-      </c>
+      <c r="O319" s="4"/>
       <c r="P319" s="4">
         <v>4500</v>
       </c>
@@ -22835,9 +22825,7 @@
       <c r="N320" s="2">
         <v>650</v>
       </c>
-      <c r="O320" s="2">
-        <v>0</v>
-      </c>
+      <c r="O320" s="2"/>
       <c r="P320" s="2">
         <v>2000</v>
       </c>
@@ -22894,9 +22882,7 @@
       <c r="N321" s="4">
         <v>630</v>
       </c>
-      <c r="O321" s="4">
-        <v>0</v>
-      </c>
+      <c r="O321" s="4"/>
       <c r="P321" s="4">
         <v>4500</v>
       </c>
@@ -22953,9 +22939,7 @@
       <c r="N322" s="2">
         <v>650</v>
       </c>
-      <c r="O322" s="2">
-        <v>0</v>
-      </c>
+      <c r="O322" s="2"/>
       <c r="P322" s="2">
         <v>4500</v>
       </c>
@@ -23012,9 +22996,7 @@
       <c r="N323" s="4">
         <v>650</v>
       </c>
-      <c r="O323" s="4">
-        <v>0</v>
-      </c>
+      <c r="O323" s="4"/>
       <c r="P323" s="4">
         <v>4500</v>
       </c>
@@ -23071,9 +23053,7 @@
       <c r="N324" s="2">
         <v>300</v>
       </c>
-      <c r="O324" s="2">
-        <v>0</v>
-      </c>
+      <c r="O324" s="2"/>
       <c r="P324" s="2">
         <v>2000</v>
       </c>
@@ -23130,9 +23110,7 @@
       <c r="N325" s="4">
         <v>280</v>
       </c>
-      <c r="O325" s="4">
-        <v>0</v>
-      </c>
+      <c r="O325" s="4"/>
       <c r="P325" s="4">
         <v>4500</v>
       </c>
@@ -23189,9 +23167,7 @@
       <c r="N326" s="2">
         <v>300</v>
       </c>
-      <c r="O326" s="2">
-        <v>0</v>
-      </c>
+      <c r="O326" s="2"/>
       <c r="P326" s="2">
         <v>4500</v>
       </c>
@@ -23248,9 +23224,7 @@
       <c r="N327" s="4">
         <v>300</v>
       </c>
-      <c r="O327" s="4">
-        <v>0</v>
-      </c>
+      <c r="O327" s="4"/>
       <c r="P327" s="4">
         <v>4500</v>
       </c>
@@ -23307,9 +23281,7 @@
       <c r="N328" s="2">
         <v>220</v>
       </c>
-      <c r="O328" s="2">
-        <v>0</v>
-      </c>
+      <c r="O328" s="2"/>
       <c r="P328" s="2">
         <v>2000</v>
       </c>
@@ -23366,9 +23338,7 @@
       <c r="N329" s="4">
         <v>300</v>
       </c>
-      <c r="O329" s="4">
-        <v>0</v>
-      </c>
+      <c r="O329" s="4"/>
       <c r="P329" s="4">
         <v>2000</v>
       </c>
@@ -23425,9 +23395,7 @@
       <c r="N330" s="2">
         <v>300</v>
       </c>
-      <c r="O330" s="2">
-        <v>0</v>
-      </c>
+      <c r="O330" s="2"/>
       <c r="P330" s="2">
         <v>2000</v>
       </c>
@@ -23484,9 +23452,7 @@
       <c r="N331" s="4">
         <v>300</v>
       </c>
-      <c r="O331" s="4">
-        <v>0</v>
-      </c>
+      <c r="O331" s="4"/>
       <c r="P331" s="4">
         <v>4000</v>
       </c>
@@ -23543,9 +23509,7 @@
       <c r="N332" s="2">
         <v>300</v>
       </c>
-      <c r="O332" s="2">
-        <v>0</v>
-      </c>
+      <c r="O332" s="2"/>
       <c r="P332" s="2">
         <v>2000</v>
       </c>
@@ -23602,9 +23566,7 @@
       <c r="N333" s="4">
         <v>310</v>
       </c>
-      <c r="O333" s="4">
-        <v>0</v>
-      </c>
+      <c r="O333" s="4"/>
       <c r="P333" s="4">
         <v>2000</v>
       </c>
@@ -23661,9 +23623,7 @@
       <c r="N334" s="2">
         <v>310</v>
       </c>
-      <c r="O334" s="2">
-        <v>0</v>
-      </c>
+      <c r="O334" s="2"/>
       <c r="P334" s="2">
         <v>4500</v>
       </c>
@@ -23720,9 +23680,7 @@
       <c r="N335" s="4">
         <v>310</v>
       </c>
-      <c r="O335" s="4">
-        <v>0</v>
-      </c>
+      <c r="O335" s="4"/>
       <c r="P335" s="4">
         <v>4000</v>
       </c>
@@ -23779,9 +23737,7 @@
       <c r="N336" s="2">
         <v>300</v>
       </c>
-      <c r="O336" s="2">
-        <v>0</v>
-      </c>
+      <c r="O336" s="2"/>
       <c r="P336" s="2">
         <v>2000</v>
       </c>

</xml_diff>